<commit_message>
Add infographic draft for Dynamic Header Detection and include new screenshot
</commit_message>
<xml_diff>
--- a/TipsAndTricks/DynamicHeaderRow/Data_DynamicHeaderRow - Copy.xlsx
+++ b/TipsAndTricks/DynamicHeaderRow/Data_DynamicHeaderRow - Copy.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="37" documentId="11_F25DC773A252ABDACC104844019D7F725BDE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D68731A-E84C-4AFE-AE8A-0F630BBBD707}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -129,6 +129,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -538,301 +542,301 @@
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
         <f t="shared" ref="A7:G16" ca="1" si="0">RANDBETWEEN(20,100)</f>
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="B7">
         <f t="shared" ca="1" si="0"/>
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C7">
         <f t="shared" ca="1" si="0"/>
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="D7">
         <f t="shared" ca="1" si="0"/>
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E7">
         <f t="shared" ca="1" si="0"/>
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="F7">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>93</v>
       </c>
       <c r="G7">
         <f t="shared" ca="1" si="0"/>
-        <v>68</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <f t="shared" ca="1" si="0"/>
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="B8">
         <f t="shared" ca="1" si="0"/>
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="C8">
         <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="D8">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="E8">
         <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="F8">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="G8">
         <f t="shared" ca="1" si="0"/>
-        <v>53</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
         <f t="shared" ca="1" si="0"/>
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B9">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="C9">
         <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D9">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E9">
         <f t="shared" ca="1" si="0"/>
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="F9">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="G9">
         <f t="shared" ca="1" si="0"/>
-        <v>51</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="B10">
         <f t="shared" ca="1" si="0"/>
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="C10">
         <f t="shared" ca="1" si="0"/>
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="D10">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="E10">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="F10">
         <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="G10">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <f t="shared" ca="1" si="0"/>
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <f t="shared" ca="1" si="0"/>
+        <v>99</v>
+      </c>
+      <c r="C11">
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="D11">
+        <f t="shared" ca="1" si="0"/>
+        <v>93</v>
+      </c>
+      <c r="E11">
+        <f t="shared" ca="1" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="F11">
+        <f t="shared" ca="1" si="0"/>
         <v>21</v>
       </c>
-      <c r="C11">
-        <f t="shared" ca="1" si="0"/>
-        <v>58</v>
-      </c>
-      <c r="D11">
-        <f t="shared" ca="1" si="0"/>
-        <v>44</v>
-      </c>
-      <c r="E11">
-        <f t="shared" ca="1" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="F11">
-        <f t="shared" ca="1" si="0"/>
-        <v>53</v>
-      </c>
       <c r="G11">
         <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="B12">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C12">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="D12">
         <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="E12">
         <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="F12">
         <f t="shared" ca="1" si="0"/>
+        <v>69</v>
+      </c>
+      <c r="G12">
+        <f t="shared" ca="1" si="0"/>
         <v>91</v>
-      </c>
-      <c r="G12">
-        <f t="shared" ca="1" si="0"/>
-        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="B13">
         <f t="shared" ca="1" si="0"/>
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="C13">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="D13">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E13">
         <f t="shared" ca="1" si="0"/>
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="F13">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="0"/>
-        <v>59</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <f t="shared" ca="1" si="0"/>
+        <v>68</v>
+      </c>
+      <c r="B14">
+        <f t="shared" ca="1" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="C14">
+        <f t="shared" ca="1" si="0"/>
+        <v>59</v>
+      </c>
+      <c r="D14">
+        <f t="shared" ca="1" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="E14">
+        <f t="shared" ca="1" si="0"/>
+        <v>62</v>
+      </c>
+      <c r="F14">
+        <f t="shared" ca="1" si="0"/>
         <v>43</v>
       </c>
-      <c r="B14">
-        <f t="shared" ca="1" si="0"/>
-        <v>33</v>
-      </c>
-      <c r="C14">
-        <f t="shared" ca="1" si="0"/>
-        <v>73</v>
-      </c>
-      <c r="D14">
-        <f t="shared" ca="1" si="0"/>
-        <v>88</v>
-      </c>
-      <c r="E14">
-        <f t="shared" ca="1" si="0"/>
-        <v>90</v>
-      </c>
-      <c r="F14">
-        <f t="shared" ca="1" si="0"/>
-        <v>57</v>
-      </c>
       <c r="G14">
         <f t="shared" ca="1" si="0"/>
-        <v>59</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
         <f t="shared" ca="1" si="0"/>
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B15">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="C15">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="D15">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="E15">
         <f t="shared" ca="1" si="0"/>
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="F15">
         <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="G15">
         <f t="shared" ca="1" si="0"/>
-        <v>53</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="B16">
         <f t="shared" ca="1" si="0"/>
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="C16">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="D16">
         <f t="shared" ca="1" si="0"/>
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E16">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F16">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="G16">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -940,301 +944,301 @@
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
         <f t="shared" ref="A5:G14" ca="1" si="0">RANDBETWEEN(20,100)</f>
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="B5">
         <f t="shared" ca="1" si="0"/>
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C5">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>41</v>
       </c>
       <c r="D5">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="E5">
         <f t="shared" ca="1" si="0"/>
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="F5">
         <f t="shared" ca="1" si="0"/>
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="G5">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="B6">
         <f t="shared" ca="1" si="0"/>
-        <v>50</v>
+        <v>86</v>
       </c>
       <c r="C6">
         <f t="shared" ca="1" si="0"/>
-        <v>69</v>
+        <v>22</v>
       </c>
       <c r="D6">
         <f t="shared" ca="1" si="0"/>
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="E6">
         <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>79</v>
       </c>
       <c r="F6">
         <f t="shared" ca="1" si="0"/>
-        <v>88</v>
+        <v>37</v>
       </c>
       <c r="G6">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B7">
         <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="C7">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="D7">
         <f t="shared" ca="1" si="0"/>
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="E7">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="F7">
         <f t="shared" ca="1" si="0"/>
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="G7">
         <f t="shared" ca="1" si="0"/>
-        <v>28</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
         <f t="shared" ca="1" si="0"/>
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B8">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="C8">
         <f t="shared" ca="1" si="0"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="D8">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E8">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="F8">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="G8">
         <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B9">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="C9">
         <f t="shared" ca="1" si="0"/>
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D9">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="E9">
         <f t="shared" ca="1" si="0"/>
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="F9">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="G9">
         <f t="shared" ca="1" si="0"/>
-        <v>42</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="B10">
         <f t="shared" ca="1" si="0"/>
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="C10">
         <f t="shared" ca="1" si="0"/>
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="D10">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="E10">
         <f t="shared" ca="1" si="0"/>
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="F10">
         <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="G10">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="B11">
         <f t="shared" ca="1" si="0"/>
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="C11">
         <f t="shared" ca="1" si="0"/>
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="D11">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="E11">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F11">
         <f t="shared" ca="1" si="0"/>
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="G11">
         <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B12">
         <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="C12">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="D12">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E12">
         <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <v>100</v>
       </c>
       <c r="F12">
         <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="G12">
         <f t="shared" ca="1" si="0"/>
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="B13">
         <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <v>84</v>
       </c>
       <c r="C13">
         <f t="shared" ca="1" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="D13">
+        <f t="shared" ca="1" si="0"/>
         <v>27</v>
       </c>
-      <c r="D13">
-        <f t="shared" ca="1" si="0"/>
-        <v>53</v>
-      </c>
       <c r="E13">
         <f t="shared" ca="1" si="0"/>
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="F13">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>37</v>
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <f t="shared" ca="1" si="0"/>
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B14">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>62</v>
       </c>
       <c r="C14">
         <f t="shared" ca="1" si="0"/>
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="D14">
         <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="E14">
         <f t="shared" ca="1" si="0"/>
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="F14">
         <f t="shared" ca="1" si="0"/>
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="G14">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1481,11 +1485,11 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <f t="shared" ref="A11:G20" ca="1" si="0">RANDBETWEEN(20,100)</f>
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="B11">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="C11">
         <f t="shared" ca="1" si="0"/>
@@ -1493,11 +1497,11 @@
       </c>
       <c r="D11">
         <f t="shared" ca="1" si="0"/>
-        <v>32</v>
+        <v>100</v>
       </c>
       <c r="E11">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="F11">
         <f t="shared" ca="1" si="0"/>
@@ -1505,277 +1509,277 @@
       </c>
       <c r="G11">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <f t="shared" ca="1" si="0"/>
+        <v>83</v>
+      </c>
+      <c r="B12">
+        <f t="shared" ca="1" si="0"/>
+        <v>69</v>
+      </c>
+      <c r="C12">
+        <f t="shared" ca="1" si="0"/>
         <v>73</v>
       </c>
-      <c r="B12">
-        <f t="shared" ca="1" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="C12">
-        <f t="shared" ca="1" si="0"/>
-        <v>100</v>
-      </c>
       <c r="D12">
         <f t="shared" ca="1" si="0"/>
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="E12">
         <f t="shared" ca="1" si="0"/>
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="F12">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>41</v>
       </c>
       <c r="G12">
         <f t="shared" ca="1" si="0"/>
-        <v>42</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <v>97</v>
       </c>
       <c r="B13">
         <f t="shared" ca="1" si="0"/>
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="C13">
         <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="D13">
         <f t="shared" ca="1" si="0"/>
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="E13">
         <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="F13">
         <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="B14">
         <f t="shared" ca="1" si="0"/>
+        <v>58</v>
+      </c>
+      <c r="C14">
+        <f t="shared" ca="1" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="D14">
+        <f t="shared" ca="1" si="0"/>
+        <v>93</v>
+      </c>
+      <c r="E14">
+        <f t="shared" ca="1" si="0"/>
         <v>87</v>
       </c>
-      <c r="C14">
-        <f t="shared" ca="1" si="0"/>
-        <v>86</v>
-      </c>
-      <c r="D14">
-        <f t="shared" ca="1" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="E14">
-        <f t="shared" ca="1" si="0"/>
-        <v>23</v>
-      </c>
       <c r="F14">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>21</v>
       </c>
       <c r="G14">
         <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="B15">
         <f t="shared" ca="1" si="0"/>
+        <v>85</v>
+      </c>
+      <c r="C15">
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="D15">
+        <f t="shared" ca="1" si="0"/>
+        <v>49</v>
+      </c>
+      <c r="E15">
+        <f t="shared" ca="1" si="0"/>
+        <v>48</v>
+      </c>
+      <c r="F15">
+        <f t="shared" ca="1" si="0"/>
         <v>35</v>
       </c>
-      <c r="C15">
-        <f t="shared" ca="1" si="0"/>
-        <v>97</v>
-      </c>
-      <c r="D15">
-        <f t="shared" ca="1" si="0"/>
-        <v>89</v>
-      </c>
-      <c r="E15">
-        <f t="shared" ca="1" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="F15">
-        <f t="shared" ca="1" si="0"/>
-        <v>39</v>
-      </c>
       <c r="G15">
         <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
         <f t="shared" ca="1" si="0"/>
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="B16">
         <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C16">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="D16">
         <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="E16">
         <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="F16">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G16">
         <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="B17">
         <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C17">
         <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="D17">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="E17">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="F17">
         <f t="shared" ca="1" si="0"/>
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="G17">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="B18">
         <f t="shared" ca="1" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="C18">
+        <f t="shared" ca="1" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="D18">
+        <f t="shared" ca="1" si="0"/>
         <v>66</v>
       </c>
-      <c r="C18">
-        <f t="shared" ca="1" si="0"/>
-        <v>52</v>
-      </c>
-      <c r="D18">
-        <f t="shared" ca="1" si="0"/>
-        <v>73</v>
-      </c>
       <c r="E18">
         <f t="shared" ca="1" si="0"/>
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="F18">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="G18">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="B19">
         <f t="shared" ca="1" si="0"/>
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="C19">
         <f t="shared" ca="1" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="D19">
+        <f t="shared" ca="1" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="E19">
+        <f t="shared" ca="1" si="0"/>
         <v>46</v>
       </c>
-      <c r="D19">
-        <f t="shared" ca="1" si="0"/>
-        <v>77</v>
-      </c>
-      <c r="E19">
-        <f t="shared" ca="1" si="0"/>
-        <v>43</v>
-      </c>
       <c r="F19">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="G19">
         <f t="shared" ca="1" si="0"/>
-        <v>66</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="B20">
         <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="C20">
         <f t="shared" ca="1" si="0"/>
-        <v>39</v>
+        <v>89</v>
       </c>
       <c r="D20">
         <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <v>89</v>
       </c>
       <c r="E20">
         <f t="shared" ca="1" si="0"/>
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="F20">
         <f t="shared" ca="1" si="0"/>
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="G20">
         <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1975,37 +1979,37 @@
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
         <f t="shared" ref="A9:G18" ca="1" si="0">RANDBETWEEN(20,100)</f>
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="B9">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C9">
         <f t="shared" ca="1" si="0"/>
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="D9">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="E9">
         <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F9">
         <f t="shared" ca="1" si="0"/>
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="G9">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
         <f t="shared" ca="1" si="0"/>
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="B10">
         <f t="shared" ca="1" si="0"/>
@@ -2013,263 +2017,263 @@
       </c>
       <c r="C10">
         <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D10">
         <f t="shared" ca="1" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="E10">
+        <f t="shared" ca="1" si="0"/>
         <v>57</v>
       </c>
-      <c r="E10">
-        <f t="shared" ca="1" si="0"/>
-        <v>44</v>
-      </c>
       <c r="F10">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G10">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B11">
         <f t="shared" ca="1" si="0"/>
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="C11">
         <f t="shared" ca="1" si="0"/>
+        <v>77</v>
+      </c>
+      <c r="D11">
+        <f t="shared" ca="1" si="0"/>
+        <v>47</v>
+      </c>
+      <c r="E11">
+        <f t="shared" ca="1" si="0"/>
         <v>22</v>
       </c>
-      <c r="D11">
-        <f t="shared" ca="1" si="0"/>
-        <v>90</v>
-      </c>
-      <c r="E11">
-        <f t="shared" ca="1" si="0"/>
-        <v>33</v>
-      </c>
       <c r="F11">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="G11">
         <f t="shared" ca="1" si="0"/>
-        <v>86</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
         <f t="shared" ca="1" si="0"/>
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="B12">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>51</v>
       </c>
       <c r="C12">
         <f t="shared" ca="1" si="0"/>
-        <v>32</v>
+        <v>77</v>
       </c>
       <c r="D12">
         <f t="shared" ca="1" si="0"/>
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E12">
         <f t="shared" ca="1" si="0"/>
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="F12">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="G12">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>39</v>
       </c>
       <c r="B13">
         <f t="shared" ca="1" si="0"/>
+        <v>67</v>
+      </c>
+      <c r="C13">
+        <f t="shared" ca="1" si="0"/>
         <v>37</v>
       </c>
-      <c r="C13">
-        <f t="shared" ca="1" si="0"/>
-        <v>34</v>
-      </c>
       <c r="D13">
         <f t="shared" ca="1" si="0"/>
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="E13">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="F13">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
         <f t="shared" ca="1" si="0"/>
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="B14">
         <f t="shared" ca="1" si="0"/>
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="C14">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D14">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>53</v>
       </c>
       <c r="E14">
         <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="F14">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="G14">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
         <f t="shared" ca="1" si="0"/>
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="B15">
         <f t="shared" ca="1" si="0"/>
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="C15">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="D15">
         <f t="shared" ca="1" si="0"/>
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="E15">
         <f t="shared" ca="1" si="0"/>
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="F15">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="G15">
         <f t="shared" ca="1" si="0"/>
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
         <f t="shared" ca="1" si="0"/>
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B16">
         <f t="shared" ca="1" si="0"/>
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C16">
         <f t="shared" ca="1" si="0"/>
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="D16">
         <f t="shared" ca="1" si="0"/>
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="E16">
         <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="F16">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="G16">
         <f t="shared" ca="1" si="0"/>
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="B17">
         <f t="shared" ca="1" si="0"/>
-        <v>59</v>
+        <v>98</v>
       </c>
       <c r="C17">
         <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <v>86</v>
       </c>
       <c r="D17">
         <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E17">
         <f t="shared" ca="1" si="0"/>
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="F17">
         <f t="shared" ca="1" si="0"/>
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="G17">
         <f t="shared" ca="1" si="0"/>
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B18">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="C18">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="D18">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E18">
         <f t="shared" ca="1" si="0"/>
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F18">
         <f t="shared" ca="1" si="0"/>
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="G18">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>